<commit_message>
Historia de Usuario 2
</commit_message>
<xml_diff>
--- a/backend/scripts/plantilla_estudiantes_ejemplo.xlsx
+++ b/backend/scripts/plantilla_estudiantes_ejemplo.xlsx
@@ -1,41 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\Downloads\PROYECTO DE GRADO 2\encuesta_proyecto-grado-2-\backend\scripts\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE470EB7-AE7A-4E18-82FE-F5F1E54B7B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Habilitados" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+  <si>
+    <t>Carnet</t>
+  </si>
+  <si>
+    <t>Nombres</t>
+  </si>
+  <si>
+    <t>Apellidos</t>
+  </si>
+  <si>
+    <t>Carrera</t>
+  </si>
+  <si>
+    <t>Modalidad</t>
+  </si>
+  <si>
+    <t>Gestion</t>
+  </si>
+  <si>
+    <t>Ingeniería de Sistemas</t>
+  </si>
+  <si>
+    <t>Proyecto de Grado</t>
+  </si>
+  <si>
+    <t>2026-1</t>
+  </si>
+  <si>
+    <t>Administración de Empresas</t>
+  </si>
+  <si>
+    <t>Tesis</t>
+  </si>
+  <si>
+    <t>Jared Neil</t>
+  </si>
+  <si>
+    <t>Pimentel Silva</t>
+  </si>
+  <si>
+    <t>Jhulianna Vitoria</t>
+  </si>
+  <si>
+    <t>Tarqui Alvarado</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -72,6 +113,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,112 +445,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="14.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.59765625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Carnet</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Nombres</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Apellidos</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Carrera</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Modalidad</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Gestion</v>
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>8492012</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Juan Carlos</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Pérez Ramos</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ingeniería de Sistemas</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Proyecto de Grado</v>
-      </c>
-      <c r="F2" t="str">
-        <v>2026-1</v>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>12926367</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>9381023</v>
-      </c>
-      <c r="B3" t="str">
-        <v>María Elena</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Gómez Flores</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Administración de Empresas</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Tesis</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-1</v>
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>12345891</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>7281944</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Rodrigo</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Mamani Quispe</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Ingeniería Industrial</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Trabajo Dirigido</v>
-      </c>
-      <c r="F4" t="str">
-        <v>2026-1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>6192840</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Camila Sofía</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Vargas Torrico</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Derecho</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Examen de Grado</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-1</v>
-      </c>
-    </row>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError sqref="A1:F1 D2:F2 D3:F3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Historia de usuario 3
</commit_message>
<xml_diff>
--- a/backend/scripts/plantilla_estudiantes_ejemplo.xlsx
+++ b/backend/scripts/plantilla_estudiantes_ejemplo.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\Downloads\PROYECTO DE GRADO 2\encuesta_proyecto-grado-2-\backend\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE470EB7-AE7A-4E18-82FE-F5F1E54B7B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7AED6C-EAE3-4321-9F03-61F6FC279D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Habilitados" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Carnet</t>
   </si>
@@ -70,6 +70,18 @@
   </si>
   <si>
     <t>Tarqui Alvarado</t>
+  </si>
+  <si>
+    <t>Carlos Ignacio</t>
+  </si>
+  <si>
+    <t>Caba Roque</t>
+  </si>
+  <si>
+    <t>Psicologia</t>
+  </si>
+  <si>
+    <t>Trabajo dirigido</t>
   </si>
 </sst>
 </file>
@@ -446,15 +458,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.09765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>12926367</v>
       </c>
@@ -494,7 +507,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>12345891</v>
       </c>
@@ -514,8 +527,26 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>98765432</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>